<commit_message>
fixed missing anchors in gblems expanded
</commit_message>
<xml_diff>
--- a/gblems_expanded.xlsx
+++ b/gblems_expanded.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ryantracy/Desktop/andre rc studies/police meta perceptions project/study 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F15DF996-2311-9E49-9910-D57CC4E72996}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01349FAC-1614-1741-99A1-546383C11839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4060" yWindow="3160" windowWidth="27240" windowHeight="16440" xr2:uid="{41654286-75BC-2243-9840-52009D08B340}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>domain</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>Extremely</t>
+  </si>
+  <si>
+    <t>Very much</t>
   </si>
 </sst>
 </file>
@@ -487,6 +490,12 @@
       <c r="B3" t="s">
         <v>9</v>
       </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">

</xml_diff>

<commit_message>
drop redundant question from gblems_expanded
</commit_message>
<xml_diff>
--- a/gblems_expanded.xlsx
+++ b/gblems_expanded.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ryantracy/Desktop/andre rc studies/police meta perceptions project/study 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01349FAC-1614-1741-99A1-546383C11839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E00B954-5FF0-A645-8641-632F9BCF82E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4060" yWindow="3160" windowWidth="27240" windowHeight="16440" xr2:uid="{41654286-75BC-2243-9840-52009D08B340}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>domain</t>
   </si>
@@ -48,18 +48,6 @@
   </si>
   <si>
     <t>maximum</t>
-  </si>
-  <si>
-    <t>perceived_intent</t>
-  </si>
-  <si>
-    <t>What is the likelihood that a police officer has ill/bad intentions towards your racial group?</t>
-  </si>
-  <si>
-    <t>Extremely unlikely</t>
-  </si>
-  <si>
-    <t>Extremely likely</t>
   </si>
   <si>
     <t>law_order</t>
@@ -452,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8A2E25F-FE4E-5549-BF60-3BAE3C59AC12}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -477,38 +465,24 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>